<commit_message>
ADD: rotas, templates, err
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr filterPrivacy="true"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD106E99-D1B7-4BE3-B382-C1698376AF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas" sheetId="1" r:id="rId1"/>
-    <sheet name="Ligar Hoje" sheetId="2" r:id="rId5"/>
+    <sheet name="Ligar Hoje" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
-  <fileRecoveryPr repairLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -48,94 +48,115 @@
     <t>MG</t>
   </si>
   <si>
+    <t>SpeedLink</t>
+  </si>
+  <si>
+    <t>Itajuba</t>
+  </si>
+  <si>
+    <t>Dita Eva</t>
+  </si>
+  <si>
+    <t>Contatado</t>
+  </si>
+  <si>
+    <t>ltraFibra</t>
+  </si>
+  <si>
+    <t>Santa Rita</t>
+  </si>
+  <si>
+    <t>Dito Moita</t>
+  </si>
+  <si>
+    <t>Juniho Play</t>
+  </si>
+  <si>
+    <t>x1</t>
+  </si>
+  <si>
+    <t>São José</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>ana</t>
+  </si>
+  <si>
+    <t>x2</t>
+  </si>
+  <si>
+    <t>Joana</t>
+  </si>
+  <si>
+    <t>x3</t>
+  </si>
+  <si>
+    <t>Taubate</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>x4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Rita </t>
+  </si>
+  <si>
+    <t>Ken</t>
+  </si>
+  <si>
+    <t>Em ligação</t>
+  </si>
+  <si>
+    <t>x5</t>
+  </si>
+  <si>
+    <t>Ryu</t>
+  </si>
+  <si>
     <t>Novo</t>
   </si>
   <si>
-    <t>SpeedLink</t>
-  </si>
-  <si>
-    <t>Itajuba</t>
-  </si>
-  <si>
-    <t>Dita Eva</t>
-  </si>
-  <si>
-    <t>Contatado</t>
-  </si>
-  <si>
-    <t>ltraFibra</t>
-  </si>
-  <si>
-    <t>Santa Rita</t>
-  </si>
-  <si>
-    <t>Dito Moita</t>
-  </si>
-  <si>
-    <t>Juniho Play</t>
-  </si>
-  <si>
-    <t>x1</t>
-  </si>
-  <si>
-    <t>São José</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>ana</t>
+    <t>35987641987</t>
+  </si>
+  <si>
+    <t>03-04-26</t>
+  </si>
+  <si>
+    <t>x6</t>
+  </si>
+  <si>
+    <t>Bela Vista</t>
+  </si>
+  <si>
+    <t>Mg</t>
+  </si>
+  <si>
+    <t>Dhalsin</t>
   </si>
   <si>
     <t>novo</t>
-  </si>
-  <si>
-    <t>x2</t>
-  </si>
-  <si>
-    <t>Joana</t>
-  </si>
-  <si>
-    <t>35999999999</t>
-  </si>
-  <si>
-    <t>03-04-26</t>
-  </si>
-  <si>
-    <t>35977777777</t>
-  </si>
-  <si>
-    <t>03-01-26</t>
-  </si>
-  <si>
-    <t>35911111111</t>
-  </si>
-  <si>
-    <t>02-01-22</t>
-  </si>
-  <si>
-    <t>35911111222</t>
-  </si>
-  <si>
-    <t>12-02-25</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -165,16 +186,16 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -187,7 +208,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -444,18 +465,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="25"/>
-    <col customWidth="true" max="3" min="2" width="15"/>
-    <col customWidth="true" max="4" min="4" width="18"/>
-    <col customWidth="true" max="5" min="5" width="24.33203125"/>
-    <col customWidth="true" max="6" min="6" width="25.77734375"/>
-    <col customWidth="true" max="7" min="7" width="20"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="6" max="6" width="25.77734375" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +499,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -492,21 +513,21 @@
         <v>35999999999</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2" s="2">
         <v>46085</v>
       </c>
       <c r="G2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -515,21 +536,21 @@
         <v>35988888888</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" s="2">
         <v>46083</v>
       </c>
       <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -538,71 +559,164 @@
         <v>35977777777</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="2">
         <v>46082</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
       </c>
       <c r="D5">
         <v>35911111111</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" s="2">
         <v>44593</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
         <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
       </c>
       <c r="D6">
         <v>35911111222</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F6" s="2">
         <v>45993</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>35912567865</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46001</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>35954987163</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46177</v>
+      </c>
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9">
+        <v>35987641987</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46085</v>
+      </c>
+      <c r="G9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10">
+        <v>35911226699</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46085</v>
+      </c>
+      <c r="G10" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -625,9 +739,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -636,87 +750,19 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
         <v>33</v>
       </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ADD: alterar status para ligado
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD106E99-D1B7-4BE3-B382-C1698376AF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="true"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas" sheetId="1" r:id="rId1"/>
@@ -16,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -39,124 +38,82 @@
     <t>Status</t>
   </si>
   <si>
-    <t>FibraNet</t>
-  </si>
-  <si>
-    <t>Pouso Alegre</t>
+    <t>x1</t>
+  </si>
+  <si>
+    <t>sadasd</t>
+  </si>
+  <si>
+    <t>asasd</t>
+  </si>
+  <si>
+    <t>fdfq</t>
+  </si>
+  <si>
+    <t>novo</t>
+  </si>
+  <si>
+    <t>asd</t>
+  </si>
+  <si>
+    <t>sas</t>
+  </si>
+  <si>
+    <t>gfh</t>
+  </si>
+  <si>
+    <t>fh</t>
+  </si>
+  <si>
+    <t>contatado</t>
+  </si>
+  <si>
+    <t>mnm</t>
+  </si>
+  <si>
+    <t>okok</t>
+  </si>
+  <si>
+    <t>ouiy</t>
+  </si>
+  <si>
+    <t>rr</t>
+  </si>
+  <si>
+    <t>Em ligação</t>
+  </si>
+  <si>
+    <t>tyut</t>
+  </si>
+  <si>
+    <t>yir</t>
   </si>
   <si>
     <t>MG</t>
   </si>
   <si>
-    <t>SpeedLink</t>
-  </si>
-  <si>
-    <t>Itajuba</t>
-  </si>
-  <si>
-    <t>Dita Eva</t>
-  </si>
-  <si>
-    <t>Contatado</t>
-  </si>
-  <si>
-    <t>ltraFibra</t>
-  </si>
-  <si>
-    <t>Santa Rita</t>
-  </si>
-  <si>
-    <t>Dito Moita</t>
-  </si>
-  <si>
-    <t>Juniho Play</t>
-  </si>
-  <si>
-    <t>x1</t>
-  </si>
-  <si>
-    <t>São José</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>ana</t>
-  </si>
-  <si>
-    <t>x2</t>
-  </si>
-  <si>
-    <t>Joana</t>
-  </si>
-  <si>
-    <t>x3</t>
-  </si>
-  <si>
-    <t>Taubate</t>
-  </si>
-  <si>
-    <t>Max</t>
-  </si>
-  <si>
-    <t>x4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Rita </t>
-  </si>
-  <si>
-    <t>Ken</t>
-  </si>
-  <si>
-    <t>Em ligação</t>
-  </si>
-  <si>
-    <t>x5</t>
-  </si>
-  <si>
-    <t>Ryu</t>
-  </si>
-  <si>
-    <t>Novo</t>
-  </si>
-  <si>
-    <t>35987641987</t>
-  </si>
-  <si>
-    <t>03-04-26</t>
-  </si>
-  <si>
-    <t>x6</t>
-  </si>
-  <si>
-    <t>Bela Vista</t>
-  </si>
-  <si>
-    <t>Mg</t>
-  </si>
-  <si>
-    <t>Dhalsin</t>
-  </si>
-  <si>
-    <t>novo</t>
+    <t>fgdfgd</t>
+  </si>
+  <si>
+    <t>Ligado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -186,16 +143,16 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -208,7 +165,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -465,18 +422,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
+    <col customWidth="true" max="3" min="2" width="15"/>
+    <col customWidth="true" max="4" min="4" width="18"/>
+    <col customWidth="true" max="5" min="5" width="22"/>
+    <col customWidth="true" max="7" min="6" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,7 +455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -510,210 +466,95 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>35999999999</v>
+        <v>456465</v>
       </c>
       <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46086</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>454656</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46086</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2">
-        <v>46085</v>
-      </c>
-      <c r="G2" t="s">
-        <v>30</v>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4">
+        <v>126</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2">
+        <v>45722</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3">
-        <v>35988888888</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46083</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4">
-        <v>35977777777</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46082</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D5">
-        <v>35911111111</v>
+        <v>54645654</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2">
-        <v>44593</v>
+        <v>46087</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6">
-        <v>35911111222</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="2">
-        <v>45993</v>
-      </c>
-      <c r="G6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>35912567865</v>
-      </c>
-      <c r="E7" t="s">
         <v>26</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46001</v>
-      </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>35954987163</v>
-      </c>
-      <c r="E8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46177</v>
-      </c>
-      <c r="G8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9">
-        <v>35987641987</v>
-      </c>
-      <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" s="2">
-        <v>46085</v>
-      </c>
-      <c r="G9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10">
-        <v>35911226699</v>
-      </c>
-      <c r="E10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="2">
-        <v>46085</v>
-      </c>
-      <c r="G10" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -739,29 +580,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" t="s">
-        <v>33</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
FIX: removendo aba ligar hoje no index.html
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr filterPrivacy="true"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4276FB61-EAFC-411F-8F36-601481CCFB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas" sheetId="1" r:id="rId1"/>
@@ -15,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -96,24 +97,69 @@
   </si>
   <si>
     <t>Ligado</t>
+  </si>
+  <si>
+    <t>sad</t>
+  </si>
+  <si>
+    <t>tru</t>
+  </si>
+  <si>
+    <t>klk</t>
+  </si>
+  <si>
+    <t>ouo</t>
+  </si>
+  <si>
+    <t>iuo</t>
+  </si>
+  <si>
+    <t>ytu</t>
+  </si>
+  <si>
+    <t>eryt</t>
+  </si>
+  <si>
+    <t>ty</t>
+  </si>
+  <si>
+    <t>kghk</t>
+  </si>
+  <si>
+    <t>nmmbmb</t>
+  </si>
+  <si>
+    <t>fgh</t>
+  </si>
+  <si>
+    <t>try</t>
+  </si>
+  <si>
+    <t>eee</t>
+  </si>
+  <si>
+    <t>sdss</t>
+  </si>
+  <si>
+    <t>fff</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -143,16 +189,16 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -165,7 +211,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -422,17 +468,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="25"/>
-    <col customWidth="true" max="3" min="2" width="15"/>
-    <col customWidth="true" max="4" min="4" width="18"/>
-    <col customWidth="true" max="5" min="5" width="22"/>
-    <col customWidth="true" max="7" min="6" width="20"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,7 +501,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -478,7 +524,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -501,7 +547,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -524,7 +570,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -547,8 +593,100 @@
         <v>26</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6">
+        <v>5846546</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46090</v>
+      </c>
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46090</v>
+      </c>
+      <c r="G7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>5465465465165</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46090</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9">
+        <v>415498</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46090</v>
+      </c>
+      <c r="G9" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
ADD: rota filtrar por status
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4276FB61-EAFC-411F-8F36-601481CCFB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="true"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas" sheetId="1" r:id="rId1"/>
@@ -147,19 +146,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -189,16 +188,16 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -211,7 +210,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -469,16 +468,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="7" width="20" customWidth="1"/>
+    <col customWidth="true" max="1" min="1" width="25"/>
+    <col customWidth="true" max="3" min="2" width="15"/>
+    <col customWidth="true" max="4" min="4" width="18"/>
+    <col customWidth="true" max="5" min="5" width="22"/>
+    <col customWidth="true" max="7" min="6" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,7 +500,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -524,7 +523,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -547,7 +546,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -570,7 +569,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -593,7 +592,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -616,7 +615,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -639,7 +638,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -662,7 +661,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -686,7 +685,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
ADD: Filtrar por nao atendeu
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="true"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="4620" yWindow="2700" windowWidth="17280" windowHeight="8988"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="56">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -141,6 +141,48 @@
   </si>
   <si>
     <t>fff</t>
+  </si>
+  <si>
+    <t>dfsdfs</t>
+  </si>
+  <si>
+    <t>hgj</t>
+  </si>
+  <si>
+    <t>jhjh</t>
+  </si>
+  <si>
+    <t>fhjf</t>
+  </si>
+  <si>
+    <t>não atendeu</t>
+  </si>
+  <si>
+    <t>Não Atendeu</t>
+  </si>
+  <si>
+    <t>xds</t>
+  </si>
+  <si>
+    <t>dsfsdf</t>
+  </si>
+  <si>
+    <t>kmlk</t>
+  </si>
+  <si>
+    <t>iupip</t>
+  </si>
+  <si>
+    <t>asdfsdf</t>
+  </si>
+  <si>
+    <t>fdgdhf</t>
+  </si>
+  <si>
+    <t>ihfigd</t>
+  </si>
+  <si>
+    <t>pop</t>
   </si>
 </sst>
 </file>
@@ -467,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col customWidth="true" max="1" min="1" width="25"/>
@@ -658,7 +700,7 @@
         <v>46090</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -681,6 +723,75 @@
         <v>46090</v>
       </c>
       <c r="G9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10">
+        <v>5465465165</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="2">
+        <v>44625</v>
+      </c>
+      <c r="G10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11">
+        <v>54564654</v>
+      </c>
+      <c r="E11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46091</v>
+      </c>
+      <c r="G11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12">
+        <v>87897</v>
+      </c>
+      <c r="E12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="2">
+        <v>46091</v>
+      </c>
+      <c r="G12" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD: criando diretorios para organizar estrutura
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -290,6 +290,21 @@
   </si>
   <si>
     <t>entrar em contato com Mariana</t>
+  </si>
+  <si>
+    <t>CassiaNet</t>
+  </si>
+  <si>
+    <t>35999965548</t>
+  </si>
+  <si>
+    <t>Cibele</t>
+  </si>
+  <si>
+    <t>Não atendeu telefone</t>
+  </si>
+  <si>
+    <t>não abriu negociação</t>
   </si>
 </sst>
 </file>
@@ -973,6 +988,35 @@
         <v>91</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ADD: quando clicar em salvar fecha janela edição
</commit_message>
<xml_diff>
--- a/controle_vendas_provedores.xlsx
+++ b/controle_vendas_provedores.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>Nome do Provedor</t>
   </si>
@@ -305,6 +305,15 @@
   </si>
   <si>
     <t>não abriu negociação</t>
+  </si>
+  <si>
+    <t>(35) 99661-5548</t>
+  </si>
+  <si>
+    <t>(35) 99772-1111</t>
+  </si>
+  <si>
+    <t>(35) 99772-1177</t>
   </si>
 </sst>
 </file>
@@ -680,19 +689,19 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
         <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
         <v>23</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
         <v>25</v>
@@ -825,13 +834,13 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
         <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G8" t="s">
         <v>38</v>

</xml_diff>